<commit_message>
feat(mambahsi): add verified 6-band conformal prediction reports, per-class coverage & summary metrics
Co-authored-by: Claude <claude@anthropic.com>
</commit_message>
<xml_diff>
--- a/Classification/mambahsi/results/uncertainty_results/conformal_reports_all_models.xlsx
+++ b/Classification/mambahsi/results/uncertainty_results/conformal_reports_all_models.xlsx
@@ -9,21 +9,21 @@
   <sheets>
     <sheet name="Summary_Compact" sheetId="1" r:id="rId1"/>
     <sheet name="Run_Config" sheetId="2" r:id="rId2"/>
-    <sheet name="Split_MambaSmall" sheetId="3" r:id="rId3"/>
-    <sheet name="ClassCond_MambaSmall" sheetId="4" r:id="rId4"/>
-    <sheet name="RC3P_MambaSmall" sheetId="5" r:id="rId5"/>
-    <sheet name="Clustered_MambaSmall" sheetId="6" r:id="rId6"/>
-    <sheet name="RAPS_MambaSmall" sheetId="7" r:id="rId7"/>
-    <sheet name="Split_MambaBase" sheetId="8" r:id="rId8"/>
-    <sheet name="ClassCond_MambaBase" sheetId="9" r:id="rId9"/>
-    <sheet name="RC3P_MambaBase" sheetId="10" r:id="rId10"/>
-    <sheet name="Clustered_MambaBase" sheetId="11" r:id="rId11"/>
-    <sheet name="RAPS_MambaBase" sheetId="12" r:id="rId12"/>
-    <sheet name="Split_MambaLarge" sheetId="13" r:id="rId13"/>
-    <sheet name="ClassCond_MambaLarge" sheetId="14" r:id="rId14"/>
-    <sheet name="RC3P_MambaLarge" sheetId="15" r:id="rId15"/>
-    <sheet name="Clustered_MambaLarge" sheetId="16" r:id="rId16"/>
-    <sheet name="RAPS_MambaLarge" sheetId="17" r:id="rId17"/>
+    <sheet name="Split_MambaHSI_Small" sheetId="3" r:id="rId3"/>
+    <sheet name="ClassCond_MambaHSI_Small" sheetId="4" r:id="rId4"/>
+    <sheet name="RC3P_MambaHSI_Small" sheetId="5" r:id="rId5"/>
+    <sheet name="Clustered_MambaHSI_Small" sheetId="6" r:id="rId6"/>
+    <sheet name="RAPS_MambaHSI_Small" sheetId="7" r:id="rId7"/>
+    <sheet name="Split_MambaHSI_Base" sheetId="8" r:id="rId8"/>
+    <sheet name="ClassCond_MambaHSI_Base" sheetId="9" r:id="rId9"/>
+    <sheet name="RC3P_MambaHSI_Base" sheetId="10" r:id="rId10"/>
+    <sheet name="Clustered_MambaHSI_Base" sheetId="11" r:id="rId11"/>
+    <sheet name="RAPS_MambaHSI_Base" sheetId="12" r:id="rId12"/>
+    <sheet name="Split_MambaHSI_Large" sheetId="13" r:id="rId13"/>
+    <sheet name="ClassCond_MambaHSI_Large" sheetId="14" r:id="rId14"/>
+    <sheet name="RC3P_MambaHSI_Large" sheetId="15" r:id="rId15"/>
+    <sheet name="Clustered_MambaHSI_Large" sheetId="16" r:id="rId16"/>
+    <sheet name="RAPS_MambaHSI_Large" sheetId="17" r:id="rId17"/>
     <sheet name="Compare_Clustered" sheetId="18" r:id="rId18"/>
     <sheet name="Compare_RAPS" sheetId="19" r:id="rId19"/>
   </sheets>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="104">
   <si>
     <t>model_name</t>
   </si>
@@ -73,13 +73,13 @@
     <t>mean_per_class_coverage</t>
   </si>
   <si>
-    <t>MambaBase</t>
-  </si>
-  <si>
-    <t>MambaLarge</t>
-  </si>
-  <si>
-    <t>MambaSmall</t>
+    <t>MambaHSI_Base</t>
+  </si>
+  <si>
+    <t>MambaHSI_Large</t>
+  </si>
+  <si>
+    <t>MambaHSI_Small</t>
   </si>
   <si>
     <t>ClassConditionalConformal</t>
@@ -151,25 +151,22 @@
     <t>timestamp_utc</t>
   </si>
   <si>
-    <t>/content/drive/My Drive/Classification/data/data.csv</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/data/ref.csv</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/mambahsi/models</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/mambahsi/results/uncertainty_results</t>
-  </si>
-  <si>
-    <t>/content/drive/My Drive/Classification/mambahsi/results</t>
-  </si>
-  <si>
-    <t>2026-07-01T09:24:51.896264+00:00</t>
-  </si>
-  <si>
-    <t>SplitConformal - MambaSmall</t>
+    <t>/kaggle/input/datasets/daneshselwal/dias-6-bands-data/k001.csv</t>
+  </si>
+  <si>
+    <t>/kaggle/input/datasets/daneshselwal/dias-6-bands-data/k002.csv</t>
+  </si>
+  <si>
+    <t>/kaggle/input</t>
+  </si>
+  <si>
+    <t>/kaggle/working/Classification/mambahsi/results/uncertainty_results</t>
+  </si>
+  <si>
+    <t>2026-10-11T12:23:46.947545+00:00</t>
+  </si>
+  <si>
+    <t>SplitConformal - MambaHSI_Small</t>
   </si>
   <si>
     <t>Summary</t>
@@ -235,7 +232,7 @@
     <t>Class Map with Uncertain Mask</t>
   </si>
   <si>
-    <t>ClassConditionalConformal - MambaSmall</t>
+    <t>ClassConditionalConformal - MambaHSI_Small</t>
   </si>
   <si>
     <t>Classwise q_hat</t>
@@ -244,7 +241,7 @@
     <t>q_hat_classconditional</t>
   </si>
   <si>
-    <t>RC3P - MambaSmall</t>
+    <t>RC3P - MambaHSI_Small</t>
   </si>
   <si>
     <t>RC3P Thresholds &amp; Limits</t>
@@ -256,7 +253,7 @@
     <t>suit_index_limit</t>
   </si>
   <si>
-    <t>ClusteredConformal - MambaSmall</t>
+    <t>ClusteredConformal - MambaHSI_Small</t>
   </si>
   <si>
     <t>Class-to-Cluster Assignment</t>
@@ -292,7 +289,7 @@
     <t>Avg Uncertainty per Class</t>
   </si>
   <si>
-    <t>RAPS - MambaSmall</t>
+    <t>RAPS - MambaHSI_Small</t>
   </si>
   <si>
     <t>RAPS Parameters</t>
@@ -307,34 +304,34 @@
     <t>k_reg</t>
   </si>
   <si>
-    <t>SplitConformal - MambaBase</t>
-  </si>
-  <si>
-    <t>ClassConditionalConformal - MambaBase</t>
-  </si>
-  <si>
-    <t>RC3P - MambaBase</t>
-  </si>
-  <si>
-    <t>ClusteredConformal - MambaBase</t>
-  </si>
-  <si>
-    <t>RAPS - MambaBase</t>
-  </si>
-  <si>
-    <t>SplitConformal - MambaLarge</t>
-  </si>
-  <si>
-    <t>ClassConditionalConformal - MambaLarge</t>
-  </si>
-  <si>
-    <t>RC3P - MambaLarge</t>
-  </si>
-  <si>
-    <t>ClusteredConformal - MambaLarge</t>
-  </si>
-  <si>
-    <t>RAPS - MambaLarge</t>
+    <t>SplitConformal - MambaHSI_Base</t>
+  </si>
+  <si>
+    <t>ClassConditionalConformal - MambaHSI_Base</t>
+  </si>
+  <si>
+    <t>RC3P - MambaHSI_Base</t>
+  </si>
+  <si>
+    <t>ClusteredConformal - MambaHSI_Base</t>
+  </si>
+  <si>
+    <t>RAPS - MambaHSI_Base</t>
+  </si>
+  <si>
+    <t>SplitConformal - MambaHSI_Large</t>
+  </si>
+  <si>
+    <t>ClassConditionalConformal - MambaHSI_Large</t>
+  </si>
+  <si>
+    <t>RC3P - MambaHSI_Large</t>
+  </si>
+  <si>
+    <t>ClusteredConformal - MambaHSI_Large</t>
+  </si>
+  <si>
+    <t>RAPS - MambaHSI_Large</t>
   </si>
   <si>
     <t>Clustered CP: 3-Model Comparison</t>
@@ -1303,7 +1300,7 @@
       <xdr:col>20</xdr:col>
       <xdr:colOff>574878</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>55145</xdr:rowOff>
+      <xdr:rowOff>58711</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1321,7 +1318,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="2476500"/>
-          <a:ext cx="12766878" cy="3484145"/>
+          <a:ext cx="12766878" cy="3487711"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1341,7 +1338,7 @@
       <xdr:col>10</xdr:col>
       <xdr:colOff>44208</xdr:colOff>
       <xdr:row>60</xdr:row>
-      <xdr:rowOff>177325</xdr:rowOff>
+      <xdr:rowOff>181211</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1359,7 +1356,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="7810500"/>
-          <a:ext cx="6140208" cy="3796825"/>
+          <a:ext cx="6140208" cy="3800711"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1384,7 +1381,7 @@
       <xdr:col>20</xdr:col>
       <xdr:colOff>574878</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>55145</xdr:rowOff>
+      <xdr:rowOff>58711</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1402,7 +1399,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="2476500"/>
-          <a:ext cx="12766878" cy="3484145"/>
+          <a:ext cx="12766878" cy="3487711"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1422,7 +1419,7 @@
       <xdr:col>10</xdr:col>
       <xdr:colOff>44208</xdr:colOff>
       <xdr:row>60</xdr:row>
-      <xdr:rowOff>177325</xdr:rowOff>
+      <xdr:rowOff>181211</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1440,7 +1437,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="7810500"/>
-          <a:ext cx="6140208" cy="3796825"/>
+          <a:ext cx="6140208" cy="3800711"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2934,28 +2931,28 @@
         <v>0.95</v>
       </c>
       <c r="D2">
-        <v>0.965661252900232</v>
+        <v>0.9661252900232019</v>
       </c>
       <c r="E2">
-        <v>0.965661252900232</v>
+        <v>0.9661252900232019</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>0.965661252900232</v>
+        <v>0.9661252900232019</v>
       </c>
       <c r="H2">
-        <v>0.03433874709976798</v>
+        <v>0.03387470997679815</v>
       </c>
       <c r="I2">
-        <v>1.523568821000026</v>
+        <v>1.550834617000021</v>
       </c>
       <c r="J2">
         <v>0.05</v>
       </c>
       <c r="M2">
-        <v>0.9652025266893595</v>
+        <v>0.9665761530629858</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2969,28 +2966,28 @@
         <v>0.95</v>
       </c>
       <c r="D3">
-        <v>0.9675174013921114</v>
+        <v>0.9647331786542923</v>
       </c>
       <c r="E3">
-        <v>0.9675174013921114</v>
+        <v>0.9647331786542923</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>0.9675174013921114</v>
+        <v>0.9647331786542923</v>
       </c>
       <c r="H3">
-        <v>0.03248259860788863</v>
+        <v>0.03526682134570765</v>
       </c>
       <c r="I3">
-        <v>2.394310539999879</v>
+        <v>1.585909466000032</v>
       </c>
       <c r="J3">
         <v>0.05</v>
       </c>
       <c r="M3">
-        <v>0.9683706040006003</v>
+        <v>0.9621669169196034</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3019,7 +3016,7 @@
         <v>0.03851508120649652</v>
       </c>
       <c r="I4">
-        <v>1.507854922999968</v>
+        <v>1.589364086999979</v>
       </c>
       <c r="J4">
         <v>0.05</v>
@@ -3054,7 +3051,7 @@
         <v>0.03526682134570765</v>
       </c>
       <c r="I5">
-        <v>6.608338046999961</v>
+        <v>6.06932012599998</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -3063,7 +3060,7 @@
         <v>4</v>
       </c>
       <c r="M5">
-        <v>0.9623736723753566</v>
+        <v>0.9635909999055944</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -3077,22 +3074,22 @@
         <v>0.95</v>
       </c>
       <c r="D6">
-        <v>0.962877030162413</v>
+        <v>0.9605568445475638</v>
       </c>
       <c r="E6">
-        <v>0.962877030162413</v>
+        <v>0.9605568445475638</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6">
-        <v>0.962877030162413</v>
+        <v>0.9605568445475638</v>
       </c>
       <c r="H6">
-        <v>0.03712296983758701</v>
+        <v>0.03944315545243619</v>
       </c>
       <c r="I6">
-        <v>7.717177898000045</v>
+        <v>7.81712743099996</v>
       </c>
       <c r="J6">
         <v>0.05</v>
@@ -3101,7 +3098,7 @@
         <v>4</v>
       </c>
       <c r="M6">
-        <v>0.9603389376701503</v>
+        <v>0.9538336327963348</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3130,7 +3127,7 @@
         <v>0.04129930394431554</v>
       </c>
       <c r="I7">
-        <v>5.802788589999864</v>
+        <v>4.06873116600002</v>
       </c>
       <c r="J7">
         <v>0.05</v>
@@ -3153,7 +3150,7 @@
         <v>0.95</v>
       </c>
       <c r="D8">
-        <v>0.9990719257540603</v>
+        <v>0.9986078886310905</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -3168,7 +3165,7 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>0.5860023100001399</v>
+        <v>0.4006909670000027</v>
       </c>
       <c r="J8">
         <v>0.05</v>
@@ -3177,7 +3174,7 @@
         <v>0.01</v>
       </c>
       <c r="M8">
-        <v>0.9994446588581278</v>
+        <v>0.9990456165596441</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3191,7 +3188,7 @@
         <v>0.95</v>
       </c>
       <c r="D9">
-        <v>0.9981438515081207</v>
+        <v>0.9990719257540603</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -3206,7 +3203,7 @@
         <v>0</v>
       </c>
       <c r="I9">
-        <v>0.3751733600001899</v>
+        <v>0.4006025649999856</v>
       </c>
       <c r="J9">
         <v>0.05</v>
@@ -3215,7 +3212,7 @@
         <v>0.01</v>
       </c>
       <c r="M9">
-        <v>0.9987309532493861</v>
+        <v>0.9994446588581278</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3244,7 +3241,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>0.3777989469999739</v>
+        <v>0.398644006999973</v>
       </c>
       <c r="J10">
         <v>0.05</v>
@@ -3282,13 +3279,13 @@
         <v>0.03201856148491879</v>
       </c>
       <c r="I11">
-        <v>1.520892143000083</v>
+        <v>1.542126383999971</v>
       </c>
       <c r="J11">
         <v>0.05</v>
       </c>
       <c r="M11">
-        <v>0.9699603485188607</v>
+        <v>0.9702030919739559</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -3302,28 +3299,28 @@
         <v>0.95</v>
       </c>
       <c r="D12">
-        <v>0.9726218097447796</v>
+        <v>0.9693735498839907</v>
       </c>
       <c r="E12">
-        <v>0.9726218097447796</v>
+        <v>0.9693735498839907</v>
       </c>
       <c r="F12">
         <v>1</v>
       </c>
       <c r="G12">
-        <v>0.9726218097447796</v>
+        <v>0.9693735498839907</v>
       </c>
       <c r="H12">
-        <v>0.02737819025522042</v>
+        <v>0.03062645011600928</v>
       </c>
       <c r="I12">
-        <v>1.89641368599996</v>
+        <v>1.579437010999982</v>
       </c>
       <c r="J12">
         <v>0.05</v>
       </c>
       <c r="M12">
-        <v>0.9721094346520412</v>
+        <v>0.9668948564027309</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -3352,7 +3349,7 @@
         <v>0.03248259860788863</v>
       </c>
       <c r="I13">
-        <v>1.472184207999817</v>
+        <v>1.551916527000003</v>
       </c>
       <c r="J13">
         <v>0.05</v>
@@ -3387,7 +3384,7 @@
         <v>0.04593967517401392</v>
       </c>
       <c r="I14">
-        <v>1.577766070000052</v>
+        <v>1.633232310999972</v>
       </c>
       <c r="J14">
         <v>0.05</v>
@@ -3407,28 +3404,28 @@
         <v>0.95</v>
       </c>
       <c r="D15">
-        <v>0.9535962877030162</v>
+        <v>0.9614849187935035</v>
       </c>
       <c r="E15">
-        <v>0.9535962877030162</v>
+        <v>0.9614849187935035</v>
       </c>
       <c r="F15">
         <v>1</v>
       </c>
       <c r="G15">
-        <v>0.9535962877030162</v>
+        <v>0.9614849187935035</v>
       </c>
       <c r="H15">
-        <v>0.04640371229698376</v>
+        <v>0.03851508120649652</v>
       </c>
       <c r="I15">
-        <v>1.943958004000024</v>
+        <v>1.550181018999979</v>
       </c>
       <c r="J15">
         <v>0.05</v>
       </c>
       <c r="M15">
-        <v>0.9281885875381766</v>
+        <v>0.9397383546804692</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -3457,7 +3454,7 @@
         <v>0.04361948955916473</v>
       </c>
       <c r="I16">
-        <v>1.60036513</v>
+        <v>1.73990850499996</v>
       </c>
       <c r="J16">
         <v>0.05</v>
@@ -3478,15 +3475,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3556,29 +3553,29 @@
         <v>0.03201856148491879</v>
       </c>
       <c r="I5">
-        <v>1.520892143000083</v>
+        <v>1.542126383999971</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9699603485188607</v>
+        <v>0.9702030919739559</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3586,7 +3583,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9726477024070022</v>
+        <v>0.9715536105032823</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -3608,7 +3605,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.946927374301676</v>
+        <v>0.9497206703910615</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -3660,18 +3657,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -3679,10 +3676,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>30521</v>
+        <v>30461</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -3690,10 +3687,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>12003</v>
+        <v>11988</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -3701,10 +3698,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>10579</v>
+        <v>10564</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -3712,10 +3709,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>2462</v>
+        <v>2451</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -3723,13 +3720,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>2717</v>
+        <v>2722</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -3737,10 +3734,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>1564</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -3748,10 +3745,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>1544</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -3759,26 +3756,26 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>39920</v>
+        <v>40031</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -3786,7 +3783,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.02629274556655947</v>
+        <v>0.02619340773865819</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -3797,7 +3794,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.0401976469952503</v>
+        <v>0.03966704375134877</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -3808,7 +3805,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.03923322189700418</v>
+        <v>0.03951186579741162</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -3819,7 +3816,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.04349969592701719</v>
+        <v>0.04223597138911861</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -3830,7 +3827,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.05963279393185839</v>
+        <v>0.06008053468530294</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -3841,7 +3838,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.03715344233616502</v>
+        <v>0.03680954350193966</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -3852,7 +3849,7 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.06640642968341104</v>
+        <v>0.06549322606410268</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -3860,12 +3857,12 @@
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -3881,15 +3878,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3959,7 +3956,7 @@
         <v>0.03526682134570765</v>
       </c>
       <c r="I5">
-        <v>6.608338046999961</v>
+        <v>6.06932012599998</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -3968,23 +3965,23 @@
         <v>4</v>
       </c>
       <c r="M5">
-        <v>0.9623736723753566</v>
+        <v>0.9635909999055944</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3992,7 +3989,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9715536105032823</v>
+        <v>0.9704595185995624</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -4036,7 +4033,7 @@
         <v>4</v>
       </c>
       <c r="B14">
-        <v>0.9615384615384616</v>
+        <v>0.9711538461538461</v>
       </c>
       <c r="C14">
         <v>104</v>
@@ -4066,15 +4063,15 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -4117,7 +4114,7 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -4138,15 +4135,15 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -4154,7 +4151,7 @@
         <v>0</v>
       </c>
       <c r="B32">
-        <v>0.03876042209363606</v>
+        <v>0.03885893983282573</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -4162,7 +4159,7 @@
         <v>1</v>
       </c>
       <c r="B33">
-        <v>0.0536935843849633</v>
+        <v>0.05402429673775477</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -4170,7 +4167,7 @@
         <v>2</v>
       </c>
       <c r="B34">
-        <v>0.0372173801621658</v>
+        <v>0.03717810475978711</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -4178,20 +4175,20 @@
         <v>3</v>
       </c>
       <c r="B35">
-        <v>0.02602641727825694</v>
+        <v>0.02592388703372295</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -4199,7 +4196,7 @@
         <v>0</v>
       </c>
       <c r="B40">
-        <v>0.9441340782122905</v>
+        <v>0.9467787114845938</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -4207,7 +4204,7 @@
         <v>1</v>
       </c>
       <c r="B41">
-        <v>0.9767441860465116</v>
+        <v>0.9825581395348837</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -4215,7 +4212,7 @@
         <v>2</v>
       </c>
       <c r="B42">
-        <v>0.967266775777414</v>
+        <v>0.9656862745098039</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -4223,20 +4220,20 @@
         <v>3</v>
       </c>
       <c r="B43">
-        <v>0.9684418145956607</v>
+        <v>0.9674556213017751</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -4244,7 +4241,7 @@
         <v>0</v>
       </c>
       <c r="B48">
-        <v>0.9726177437020811</v>
+        <v>0.9715224534501643</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -4252,10 +4249,10 @@
         <v>1</v>
       </c>
       <c r="B49">
-        <v>0.9714285714285714</v>
+        <v>0.9692982456140351</v>
       </c>
       <c r="J49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -4263,7 +4260,7 @@
         <v>2</v>
       </c>
       <c r="B50">
-        <v>0.9441340782122905</v>
+        <v>0.9467787114845938</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -4279,7 +4276,7 @@
         <v>4</v>
       </c>
       <c r="B52">
-        <v>0.9615384615384616</v>
+        <v>0.9711538461538461</v>
       </c>
     </row>
     <row r="53" spans="1:10">
@@ -4300,7 +4297,7 @@
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -4316,15 +4313,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4379,7 +4376,7 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9990719257540603</v>
+        <v>0.9986078886310905</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -4394,7 +4391,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0.5860023100001399</v>
+        <v>0.4006909670000027</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -4403,23 +4400,23 @@
         <v>0.01</v>
       </c>
       <c r="M5">
-        <v>0.9994446588581278</v>
+        <v>0.9990456165596441</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -4449,7 +4446,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9972067039106145</v>
+        <v>0.994413407821229</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -4501,18 +4498,18 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -4539,15 +4536,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4602,44 +4599,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9535962877030162</v>
+        <v>0.9614849187935035</v>
       </c>
       <c r="E5">
-        <v>0.9535962877030162</v>
+        <v>0.9614849187935035</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9535962877030162</v>
+        <v>0.9614849187935035</v>
       </c>
       <c r="H5">
-        <v>0.04640371229698376</v>
+        <v>0.03851508120649652</v>
       </c>
       <c r="I5">
-        <v>1.943958004000024</v>
+        <v>1.550181018999979</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9281885875381766</v>
+        <v>0.9397383546804692</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -4647,7 +4644,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9879649890590809</v>
+        <v>0.986870897155361</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -4658,7 +4655,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9691629955947136</v>
+        <v>0.9625550660792952</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -4669,7 +4666,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9050279329608939</v>
+        <v>0.9329608938547486</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -4680,7 +4677,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.8461538461538461</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -4691,7 +4688,7 @@
         <v>4</v>
       </c>
       <c r="B14">
-        <v>0.9807692307692307</v>
+        <v>0.9903846153846154</v>
       </c>
       <c r="C14">
         <v>104</v>
@@ -4702,7 +4699,7 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>0.9405940594059405</v>
+        <v>0.9504950495049505</v>
       </c>
       <c r="C15">
         <v>101</v>
@@ -4713,7 +4710,7 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>0.8676470588235294</v>
+        <v>0.8382352941176471</v>
       </c>
       <c r="C16">
         <v>68</v>
@@ -4721,18 +4718,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -4740,10 +4737,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>33865</v>
+        <v>34700</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -4751,10 +4748,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>11777</v>
+        <v>10917</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -4762,10 +4759,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>10640</v>
+        <v>10544</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -4773,10 +4770,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>2099</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -4784,13 +4781,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>2898</v>
+        <v>2893</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -4798,7 +4795,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
         <v>1305</v>
@@ -4809,10 +4806,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>1063</v>
+        <v>999</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -4820,35 +4817,35 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>37663</v>
+        <v>37702</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33">
-        <v>0.02846348760702344</v>
+        <v>0.02726322027469863</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -4864,15 +4861,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4927,44 +4924,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9675174013921114</v>
+        <v>0.9647331786542923</v>
       </c>
       <c r="E5">
-        <v>0.9675174013921114</v>
+        <v>0.9647331786542923</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9675174013921114</v>
+        <v>0.9647331786542923</v>
       </c>
       <c r="H5">
-        <v>0.03248259860788863</v>
+        <v>0.03526682134570765</v>
       </c>
       <c r="I5">
-        <v>2.394310539999879</v>
+        <v>1.585909466000032</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9683706040006003</v>
+        <v>0.9621669169196034</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -4994,7 +4991,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.9525139664804469</v>
+        <v>0.9497206703910615</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -5005,7 +5002,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>0.9743589743589743</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -5016,7 +5013,7 @@
         <v>4</v>
       </c>
       <c r="B14">
-        <v>0.9903846153846154</v>
+        <v>1</v>
       </c>
       <c r="C14">
         <v>104</v>
@@ -5027,7 +5024,7 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>0.9603960396039604</v>
+        <v>0.9504950495049505</v>
       </c>
       <c r="C15">
         <v>101</v>
@@ -5038,7 +5035,7 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>0.9411764705882353</v>
+        <v>0.9264705882352942</v>
       </c>
       <c r="C16">
         <v>68</v>
@@ -5046,18 +5043,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -5065,10 +5062,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>31231</v>
+        <v>31635</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -5076,10 +5073,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>11640</v>
+        <v>11250</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -5087,10 +5084,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>12185</v>
+        <v>11434</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -5098,10 +5095,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>3072</v>
+        <v>2815</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -5109,13 +5106,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>3118</v>
+        <v>3443</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -5123,10 +5120,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>1519</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -5134,10 +5131,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>1335</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -5145,23 +5142,23 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>37210</v>
+        <v>38171</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -5169,7 +5166,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.0237090293399369</v>
+        <v>0.02294705023400134</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -5177,7 +5174,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.0279565258892861</v>
+        <v>0.02856044062656105</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -5185,7 +5182,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.03644557474379073</v>
+        <v>0.03130660044345002</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -5193,7 +5190,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.08327883338037556</v>
+        <v>0.05074090612395687</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -5201,7 +5198,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.03498982567976461</v>
+        <v>0.05426428691569529</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -5209,7 +5206,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.03721069123944176</v>
+        <v>0.0273917917965949</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -5217,17 +5214,17 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.04957032764683478</v>
+        <v>0.04372929919048751</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -5243,15 +5240,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5306,44 +5303,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9726218097447796</v>
+        <v>0.9693735498839907</v>
       </c>
       <c r="E5">
-        <v>0.9726218097447796</v>
+        <v>0.9693735498839907</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.9726218097447796</v>
+        <v>0.9693735498839907</v>
       </c>
       <c r="H5">
-        <v>0.02737819025522042</v>
+        <v>0.03062645011600928</v>
       </c>
       <c r="I5">
-        <v>1.89641368599996</v>
+        <v>1.579437010999982</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9721094346520412</v>
+        <v>0.9668948564027309</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -5351,7 +5348,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.975929978118162</v>
+        <v>0.9726477024070022</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -5362,7 +5359,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9691629955947136</v>
+        <v>0.9669603524229075</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -5384,7 +5381,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>0.9935897435897436</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -5406,7 +5403,7 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>0.9603960396039604</v>
+        <v>0.9504950495049505</v>
       </c>
       <c r="C15">
         <v>101</v>
@@ -5417,7 +5414,7 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>0.9411764705882353</v>
+        <v>0.9264705882352942</v>
       </c>
       <c r="C16">
         <v>68</v>
@@ -5425,18 +5422,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -5444,10 +5441,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>31587</v>
+        <v>32066</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -5455,10 +5452,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>11777</v>
+        <v>11426</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -5466,10 +5463,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>12526</v>
+        <v>11664</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -5477,10 +5474,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>3258</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -5488,13 +5485,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>3319</v>
+        <v>3501</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -5502,10 +5499,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>1545</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -5513,10 +5510,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>1335</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -5524,26 +5521,26 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>35963</v>
+        <v>37059</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -5551,7 +5548,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.0241103181390927</v>
+        <v>0.02332979483551678</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -5562,7 +5559,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.02846348760702344</v>
+        <v>0.02945024390471607</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -5573,7 +5570,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.03911547361026557</v>
+        <v>0.03284517674605458</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -5584,7 +5581,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.1032356804495714</v>
+        <v>0.06536220679397675</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -5595,7 +5592,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.04597880899494766</v>
+        <v>0.05861187331895579</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -5606,7 +5603,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.03829117554867612</v>
+        <v>0.02861162834000497</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -5617,7 +5614,7 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.04957032764683478</v>
+        <v>0.04372929919048751</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -5625,12 +5622,12 @@
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -5646,15 +5643,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5709,22 +5706,22 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.962877030162413</v>
+        <v>0.9605568445475638</v>
       </c>
       <c r="E5">
-        <v>0.962877030162413</v>
+        <v>0.9605568445475638</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.962877030162413</v>
+        <v>0.9605568445475638</v>
       </c>
       <c r="H5">
-        <v>0.03712296983758701</v>
+        <v>0.03944315545243619</v>
       </c>
       <c r="I5">
-        <v>7.717177898000045</v>
+        <v>7.81712743099996</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -5733,23 +5730,23 @@
         <v>4</v>
       </c>
       <c r="M5">
-        <v>0.9603389376701503</v>
+        <v>0.9538336327963348</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -5757,7 +5754,7 @@
         <v>0</v>
       </c>
       <c r="B10">
-        <v>0.9846827133479212</v>
+        <v>0.986870897155361</v>
       </c>
       <c r="C10">
         <v>914</v>
@@ -5768,7 +5765,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9625550660792952</v>
+        <v>0.9427312775330396</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -5779,7 +5776,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.888268156424581</v>
+        <v>0.9106145251396648</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -5790,7 +5787,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>0.9743589743589743</v>
       </c>
       <c r="C13">
         <v>156</v>
@@ -5812,7 +5809,7 @@
         <v>5</v>
       </c>
       <c r="B15">
-        <v>0.9603960396039604</v>
+        <v>0.9504950495049505</v>
       </c>
       <c r="C15">
         <v>101</v>
@@ -5823,7 +5820,7 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>0.9264705882352942</v>
+        <v>0.9117647058823529</v>
       </c>
       <c r="C16">
         <v>68</v>
@@ -5831,15 +5828,15 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -5882,7 +5879,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -5903,15 +5900,15 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -5919,7 +5916,7 @@
         <v>0</v>
       </c>
       <c r="B32">
-        <v>0.04447773809934252</v>
+        <v>0.04047974935178489</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -5927,7 +5924,7 @@
         <v>1</v>
       </c>
       <c r="B33">
-        <v>0.02719298357944611</v>
+        <v>0.02581240220977776</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -5935,7 +5932,7 @@
         <v>2</v>
       </c>
       <c r="B34">
-        <v>0.03721069123944176</v>
+        <v>0.0273917917965949</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -5943,20 +5940,20 @@
         <v>3</v>
       </c>
       <c r="B35">
-        <v>0.08327883338037556</v>
+        <v>0.05074090612395687</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -5964,7 +5961,7 @@
         <v>0</v>
       </c>
       <c r="B40">
-        <v>0.9709302325581395</v>
+        <v>0.9651162790697675</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -5972,7 +5969,7 @@
         <v>1</v>
       </c>
       <c r="B41">
-        <v>0.9594202898550724</v>
+        <v>0.9594438006952491</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -5980,7 +5977,7 @@
         <v>2</v>
       </c>
       <c r="B42">
-        <v>0.9603960396039604</v>
+        <v>0.9504950495049505</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -5988,20 +5985,20 @@
         <v>3</v>
       </c>
       <c r="B43">
-        <v>0.9936305732484076</v>
+        <v>0.9743589743589743</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -6009,7 +6006,7 @@
         <v>0</v>
       </c>
       <c r="B48">
-        <v>0.9857612267250822</v>
+        <v>0.9879518072289156</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -6017,10 +6014,10 @@
         <v>1</v>
       </c>
       <c r="B49">
-        <v>0.9604395604395605</v>
+        <v>0.9406593406593406</v>
       </c>
       <c r="J49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -6028,7 +6025,7 @@
         <v>2</v>
       </c>
       <c r="B50">
-        <v>0.8907563025210085</v>
+        <v>0.9106145251396648</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -6036,7 +6033,7 @@
         <v>3</v>
       </c>
       <c r="B51">
-        <v>0.9936305732484076</v>
+        <v>0.9743589743589743</v>
       </c>
     </row>
     <row r="52" spans="1:10">
@@ -6052,7 +6049,7 @@
         <v>5</v>
       </c>
       <c r="B53">
-        <v>0.9603960396039604</v>
+        <v>0.9504950495049505</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -6060,12 +6057,12 @@
         <v>6</v>
       </c>
       <c r="B54">
-        <v>0.9264705882352942</v>
+        <v>0.9117647058823529</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -6081,15 +6078,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -6144,7 +6141,7 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9981438515081207</v>
+        <v>0.9990719257540603</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -6159,7 +6156,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0.3751733600001899</v>
+        <v>0.4006025649999856</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -6168,23 +6165,23 @@
         <v>0.01</v>
       </c>
       <c r="M5">
-        <v>0.9987309532493861</v>
+        <v>0.9994446588581278</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -6203,7 +6200,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>0.9977973568281938</v>
+        <v>1</v>
       </c>
       <c r="C11">
         <v>454</v>
@@ -6214,7 +6211,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>0.994413407821229</v>
+        <v>0.9972067039106145</v>
       </c>
       <c r="C12">
         <v>358</v>
@@ -6266,18 +6263,18 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -6304,7 +6301,7 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6377,13 +6374,13 @@
         <v>13</v>
       </c>
       <c r="J4">
-        <v>0.9623736723753566</v>
+        <v>0.9635909999055945</v>
       </c>
       <c r="L4">
         <v>4</v>
       </c>
       <c r="M4">
-        <v>0.9623736723753566</v>
+        <v>0.9635909999055944</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -6397,31 +6394,31 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.962877030162413</v>
+        <v>0.9605568445475638</v>
       </c>
       <c r="E5">
-        <v>0.962877030162413</v>
+        <v>0.9605568445475638</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.962877030162413</v>
+        <v>0.9605568445475638</v>
       </c>
       <c r="H5">
-        <v>0.03712296983758701</v>
+        <v>0.03944315545243619</v>
       </c>
       <c r="I5" t="s">
         <v>14</v>
       </c>
       <c r="J5">
-        <v>0.9603389376701503</v>
+        <v>0.9538336327963347</v>
       </c>
       <c r="L5">
         <v>4</v>
       </c>
       <c r="M5">
-        <v>0.9603389376701503</v>
+        <v>0.9538336327963348</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -6464,12 +6461,12 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -6485,7 +6482,7 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6540,7 +6537,7 @@
         <v>0.95</v>
       </c>
       <c r="D4">
-        <v>0.9990719257540603</v>
+        <v>0.9986078886310905</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -6558,13 +6555,13 @@
         <v>13</v>
       </c>
       <c r="J4">
-        <v>0.9994446588581278</v>
+        <v>0.9990456165596441</v>
       </c>
       <c r="K4">
         <v>0.01</v>
       </c>
       <c r="M4">
-        <v>0.9994446588581278</v>
+        <v>0.9990456165596441</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -6578,7 +6575,7 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.9981438515081207</v>
+        <v>0.9990719257540603</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -6596,13 +6593,13 @@
         <v>14</v>
       </c>
       <c r="J5">
-        <v>0.9987309532493861</v>
+        <v>0.9994446588581278</v>
       </c>
       <c r="K5">
         <v>0.01</v>
       </c>
       <c r="M5">
-        <v>0.9987309532493861</v>
+        <v>0.9994446588581278</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -6645,12 +6642,12 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -6717,7 +6714,7 @@
         <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -6813,7 +6810,7 @@
         <v>38</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -6828,15 +6825,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -6906,7 +6903,7 @@
         <v>0.04361948955916473</v>
       </c>
       <c r="I5">
-        <v>1.60036513</v>
+        <v>1.73990850499996</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -6917,18 +6914,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -7010,18 +7007,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -7029,7 +7026,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
         <v>34845</v>
@@ -7040,7 +7037,7 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
         <v>10277</v>
@@ -7051,7 +7048,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
         <v>10907</v>
@@ -7062,7 +7059,7 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
         <v>2675</v>
@@ -7073,13 +7070,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
         <v>2382</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -7087,7 +7084,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
         <v>2135</v>
@@ -7098,7 +7095,7 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
         <v>1780</v>
@@ -7109,7 +7106,7 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
         <v>36309</v>
@@ -7117,27 +7114,27 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33">
-        <v>0.06771161943684512</v>
+        <v>0.06771149393264853</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -7153,15 +7150,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -7231,7 +7228,7 @@
         <v>0.03851508120649652</v>
       </c>
       <c r="I5">
-        <v>1.507854922999968</v>
+        <v>1.589364086999979</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -7242,18 +7239,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -7335,18 +7332,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -7354,7 +7351,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
         <v>31688</v>
@@ -7365,10 +7362,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>12506</v>
+        <v>12507</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -7376,7 +7373,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
         <v>11910</v>
@@ -7387,7 +7384,7 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
         <v>3959</v>
@@ -7398,13 +7395,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
         <v>2724</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -7412,10 +7409,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>1800</v>
+        <v>1801</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -7423,10 +7420,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>2322</v>
+        <v>2323</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -7434,23 +7431,23 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>34401</v>
+        <v>34398</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -7458,7 +7455,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.03692061826001236</v>
+        <v>0.0369206220719972</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -7466,7 +7463,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.1434629997771731</v>
+        <v>0.1434629713319994</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -7474,7 +7471,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.09871378248419249</v>
+        <v>0.09871372528470435</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -7482,7 +7479,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.2609392537054787</v>
+        <v>0.2609392512964148</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -7490,7 +7487,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.1234579267940122</v>
+        <v>0.1234577463358316</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -7498,7 +7495,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.04223248833197224</v>
+        <v>0.04223251633523439</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -7506,17 +7503,17 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.2183039088283467</v>
+        <v>0.2183037637746523</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -7532,15 +7529,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -7610,7 +7607,7 @@
         <v>0.03248259860788863</v>
       </c>
       <c r="I5">
-        <v>1.472184207999817</v>
+        <v>1.551916527000003</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -7621,18 +7618,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -7714,18 +7711,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -7733,10 +7730,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>31954</v>
+        <v>31953</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -7744,7 +7741,7 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
         <v>12786</v>
@@ -7755,7 +7752,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
         <v>12856</v>
@@ -7766,7 +7763,7 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
         <v>3967</v>
@@ -7777,13 +7774,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
         <v>3301</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -7791,7 +7788,7 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
         <v>1863</v>
@@ -7802,10 +7799,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>2322</v>
+        <v>2323</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -7813,7 +7810,7 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
         <v>32261</v>
@@ -7821,18 +7818,18 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -7840,7 +7837,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.03855945224394042</v>
+        <v>0.03855948661301301</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -7851,7 +7848,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.1557797611732137</v>
+        <v>0.1557799392946331</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -7862,7 +7859,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.1410650190952359</v>
+        <v>0.1410649058855332</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -7873,7 +7870,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.2618712228059514</v>
+        <v>0.2618718999090223</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -7884,7 +7881,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.2580876293304981</v>
+        <v>0.2580879940500707</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -7895,7 +7892,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.04632879415160951</v>
+        <v>0.04632885042559209</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -7906,7 +7903,7 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.2183039088283467</v>
+        <v>0.2183037637746523</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -7914,12 +7911,12 @@
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -7935,15 +7932,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -8013,7 +8010,7 @@
         <v>0.04129930394431554</v>
       </c>
       <c r="I5">
-        <v>5.802788589999864</v>
+        <v>4.06873116600002</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -8027,18 +8024,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -8120,15 +8117,15 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -8171,7 +8168,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -8192,15 +8189,15 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -8208,7 +8205,7 @@
         <v>0</v>
       </c>
       <c r="B32">
-        <v>0.0398465410622475</v>
+        <v>0.03984653715006747</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -8216,7 +8213,7 @@
         <v>1</v>
       </c>
       <c r="B33">
-        <v>0.1434629997771731</v>
+        <v>0.1434629713319994</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -8224,7 +8221,7 @@
         <v>2</v>
       </c>
       <c r="B34">
-        <v>0.09311502523952331</v>
+        <v>0.09311470834470459</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -8232,20 +8229,20 @@
         <v>3</v>
       </c>
       <c r="B35">
-        <v>0.09633443730416213</v>
+        <v>0.0963340809827643</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -8282,15 +8279,15 @@
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -8309,7 +8306,7 @@
         <v>0.9517543859649122</v>
       </c>
       <c r="J49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -8354,7 +8351,7 @@
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -8370,15 +8367,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -8448,7 +8445,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0.3777989469999739</v>
+        <v>0.398644006999973</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -8462,18 +8459,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -8555,18 +8552,18 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -8593,15 +8590,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -8671,7 +8668,7 @@
         <v>0.04593967517401392</v>
       </c>
       <c r="I5">
-        <v>1.577766070000052</v>
+        <v>1.633232310999972</v>
       </c>
       <c r="J5">
         <v>0.05</v>
@@ -8682,18 +8679,18 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -8775,18 +8772,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -8794,10 +8791,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>33159</v>
+        <v>33173</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -8805,10 +8802,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>10932</v>
+        <v>10969</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -8816,10 +8813,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>9303</v>
+        <v>9271</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -8827,10 +8824,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>2206</v>
+        <v>2213</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -8838,13 +8835,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>2206</v>
+        <v>2213</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -8852,10 +8849,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>1448</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -8863,7 +8860,7 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
         <v>1186</v>
@@ -8874,35 +8871,35 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>40870</v>
+        <v>40840</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33">
-        <v>0.03141787162345611</v>
+        <v>0.03144951208062308</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -8918,15 +8915,15 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -8981,44 +8978,44 @@
         <v>0.95</v>
       </c>
       <c r="D5">
-        <v>0.965661252900232</v>
+        <v>0.9661252900232019</v>
       </c>
       <c r="E5">
-        <v>0.965661252900232</v>
+        <v>0.9661252900232019</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0.965661252900232</v>
+        <v>0.9661252900232019</v>
       </c>
       <c r="H5">
-        <v>0.03433874709976798</v>
+        <v>0.03387470997679815</v>
       </c>
       <c r="I5">
-        <v>1.523568821000026</v>
+        <v>1.550834617000021</v>
       </c>
       <c r="J5">
         <v>0.05</v>
       </c>
       <c r="M5">
-        <v>0.9652025266893595</v>
+        <v>0.9665761530629858</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -9070,7 +9067,7 @@
         <v>4</v>
       </c>
       <c r="B14">
-        <v>0.9615384615384616</v>
+        <v>0.9711538461538461</v>
       </c>
       <c r="C14">
         <v>104</v>
@@ -9100,18 +9097,18 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -9119,10 +9116,10 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21">
-        <v>30330</v>
+        <v>30366</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -9130,10 +9127,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C22">
-        <v>11700</v>
+        <v>11737</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -9141,10 +9138,10 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23">
-        <v>10496</v>
+        <v>10478</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -9152,10 +9149,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24">
-        <v>2460</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -9163,13 +9160,13 @@
         <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25">
-        <v>2644</v>
+        <v>2651</v>
       </c>
       <c r="J25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -9177,10 +9174,10 @@
         <v>5</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26">
-        <v>1386</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -9188,10 +9185,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
-        <v>1544</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -9199,23 +9196,23 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28">
-        <v>40750</v>
+        <v>40724</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -9223,7 +9220,7 @@
         <v>0</v>
       </c>
       <c r="B33">
-        <v>0.02605987191548353</v>
+        <v>0.02605405323426357</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -9231,7 +9228,7 @@
         <v>1</v>
       </c>
       <c r="B34">
-        <v>0.0372173801621658</v>
+        <v>0.03717810475978711</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -9239,7 +9236,7 @@
         <v>2</v>
       </c>
       <c r="B35">
-        <v>0.03876042209363606</v>
+        <v>0.03885893983282573</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -9247,7 +9244,7 @@
         <v>3</v>
       </c>
       <c r="B36">
-        <v>0.04346094029492076</v>
+        <v>0.04092546907547989</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -9255,7 +9252,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>0.0536935843849633</v>
+        <v>0.05402429673775477</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -9263,7 +9260,7 @@
         <v>5</v>
       </c>
       <c r="B38">
-        <v>0.02877599892226801</v>
+        <v>0.0292987960117258</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -9271,17 +9268,17 @@
         <v>6</v>
       </c>
       <c r="B39">
-        <v>0.06640642968341104</v>
+        <v>0.06549322606410268</v>
       </c>
     </row>
     <row r="49" spans="10:10">
       <c r="J49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="10:10">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>